<commit_message>
Fix: Resolution Timeout HTTP via configuration Security Group (Port 80)
</commit_message>
<xml_diff>
--- a/Feuille de calcul de la base de connaissance-1.xlsx
+++ b/Feuille de calcul de la base de connaissance-1.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Anna\Documents\ODC\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{97BB696F-C9C9-4675-AFF3-A595EDA0F9B9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E3742529-D561-49A7-8D9F-A635011B9630}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -671,38 +671,38 @@
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="6" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -1189,106 +1189,106 @@
       </c>
     </row>
     <row r="6" spans="1:9" ht="40.5" customHeight="1">
-      <c r="A6" s="30" t="s">
+      <c r="A6" s="29" t="s">
         <v>48</v>
       </c>
-      <c r="B6" s="25" t="s">
+      <c r="B6" s="32" t="s">
         <v>47</v>
       </c>
-      <c r="C6" s="27" t="s">
+      <c r="C6" s="34" t="s">
         <v>50</v>
       </c>
-      <c r="D6" s="29" t="s">
+      <c r="D6" s="26" t="s">
         <v>51</v>
       </c>
-      <c r="E6" s="29" t="s">
+      <c r="E6" s="26" t="s">
         <v>52</v>
       </c>
-      <c r="F6" s="29" t="s">
+      <c r="F6" s="26" t="s">
         <v>53</v>
       </c>
-      <c r="G6" s="29" t="s">
+      <c r="G6" s="26" t="s">
         <v>54</v>
       </c>
-      <c r="H6" s="29" t="s">
+      <c r="H6" s="26" t="s">
         <v>55</v>
       </c>
-      <c r="I6" s="32" t="s">
+      <c r="I6" s="27" t="s">
         <v>49</v>
       </c>
     </row>
     <row r="7" spans="1:9" ht="40" customHeight="1">
-      <c r="A7" s="31"/>
-      <c r="B7" s="24"/>
-      <c r="C7" s="26"/>
-      <c r="D7" s="28"/>
-      <c r="E7" s="28"/>
-      <c r="F7" s="28"/>
-      <c r="G7" s="28"/>
-      <c r="H7" s="28"/>
-      <c r="I7" s="33"/>
+      <c r="A7" s="30"/>
+      <c r="B7" s="33"/>
+      <c r="C7" s="31"/>
+      <c r="D7" s="24"/>
+      <c r="E7" s="24"/>
+      <c r="F7" s="24"/>
+      <c r="G7" s="24"/>
+      <c r="H7" s="24"/>
+      <c r="I7" s="28"/>
     </row>
     <row r="8" spans="1:9" ht="40" customHeight="1">
-      <c r="A8" s="31"/>
-      <c r="B8" s="24"/>
-      <c r="C8" s="26"/>
-      <c r="D8" s="28"/>
-      <c r="E8" s="28"/>
-      <c r="F8" s="28"/>
-      <c r="G8" s="28"/>
-      <c r="H8" s="28"/>
-      <c r="I8" s="33"/>
+      <c r="A8" s="30"/>
+      <c r="B8" s="33"/>
+      <c r="C8" s="31"/>
+      <c r="D8" s="24"/>
+      <c r="E8" s="24"/>
+      <c r="F8" s="24"/>
+      <c r="G8" s="24"/>
+      <c r="H8" s="24"/>
+      <c r="I8" s="28"/>
     </row>
     <row r="9" spans="1:9" ht="40" customHeight="1">
-      <c r="A9" s="34" t="s">
+      <c r="A9" s="25" t="s">
         <v>64</v>
       </c>
-      <c r="B9" s="26" t="s">
+      <c r="B9" s="31" t="s">
         <v>57</v>
       </c>
-      <c r="C9" s="26" t="s">
+      <c r="C9" s="31" t="s">
         <v>56</v>
       </c>
-      <c r="D9" s="28" t="s">
+      <c r="D9" s="24" t="s">
         <v>59</v>
       </c>
-      <c r="E9" s="28" t="s">
+      <c r="E9" s="24" t="s">
         <v>60</v>
       </c>
-      <c r="F9" s="28" t="s">
+      <c r="F9" s="24" t="s">
         <v>58</v>
       </c>
-      <c r="G9" s="28" t="s">
+      <c r="G9" s="24" t="s">
         <v>61</v>
       </c>
-      <c r="H9" s="28" t="s">
+      <c r="H9" s="24" t="s">
         <v>62</v>
       </c>
-      <c r="I9" s="28" t="s">
+      <c r="I9" s="24" t="s">
         <v>63</v>
       </c>
     </row>
     <row r="10" spans="1:9" ht="22.5" customHeight="1">
-      <c r="A10" s="34"/>
-      <c r="B10" s="26"/>
-      <c r="C10" s="26"/>
-      <c r="D10" s="28"/>
-      <c r="E10" s="28"/>
-      <c r="F10" s="28"/>
-      <c r="G10" s="28"/>
-      <c r="H10" s="28"/>
-      <c r="I10" s="28"/>
+      <c r="A10" s="25"/>
+      <c r="B10" s="31"/>
+      <c r="C10" s="31"/>
+      <c r="D10" s="24"/>
+      <c r="E10" s="24"/>
+      <c r="F10" s="24"/>
+      <c r="G10" s="24"/>
+      <c r="H10" s="24"/>
+      <c r="I10" s="24"/>
     </row>
     <row r="11" spans="1:9" ht="22.5" customHeight="1">
-      <c r="A11" s="34"/>
-      <c r="B11" s="26"/>
-      <c r="C11" s="26"/>
-      <c r="D11" s="28"/>
-      <c r="E11" s="28"/>
-      <c r="F11" s="28"/>
-      <c r="G11" s="28"/>
-      <c r="H11" s="28"/>
-      <c r="I11" s="28"/>
+      <c r="A11" s="25"/>
+      <c r="B11" s="31"/>
+      <c r="C11" s="31"/>
+      <c r="D11" s="24"/>
+      <c r="E11" s="24"/>
+      <c r="F11" s="24"/>
+      <c r="G11" s="24"/>
+      <c r="H11" s="24"/>
+      <c r="I11" s="24"/>
     </row>
     <row r="12" spans="1:9" ht="22.5">
       <c r="A12" s="4"/>
@@ -1817,6 +1817,8 @@
     </row>
   </sheetData>
   <mergeCells count="18">
+    <mergeCell ref="F6:F8"/>
+    <mergeCell ref="G6:G8"/>
     <mergeCell ref="H9:H11"/>
     <mergeCell ref="I9:I11"/>
     <mergeCell ref="A9:A11"/>
@@ -1833,8 +1835,6 @@
     <mergeCell ref="C6:C8"/>
     <mergeCell ref="D6:D8"/>
     <mergeCell ref="E6:E8"/>
-    <mergeCell ref="F6:F8"/>
-    <mergeCell ref="G6:G8"/>
   </mergeCells>
   <phoneticPr fontId="13" type="noConversion"/>
   <dataValidations count="1">
@@ -1901,21 +1901,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Dokument" ma:contentTypeID="0x01010006807B066C556C4DA1F97EE96CC1104B" ma:contentTypeVersion="13" ma:contentTypeDescription="Utwórz nowy dokument." ma:contentTypeScope="" ma:versionID="cfb987611df5cdae7f7a5067c3395bc7">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="c2ee6f6c-285d-4b95-ace0-9682ebe56039" xmlns:ns3="012b183d-1ada-4ff6-b855-98c4d59bda2b" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="08f2586826dc5d0b05e832f2b79fc23a" ns2:_="" ns3:_="">
     <xsd:import namespace="c2ee6f6c-285d-4b95-ace0-9682ebe56039"/>
@@ -2138,10 +2123,36 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C795275D-8D89-4504-820D-42600FA03DDE}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E55E6835-5439-4B85-9C34-8A416D678E4C}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="c2ee6f6c-285d-4b95-ace0-9682ebe56039"/>
+    <ds:schemaRef ds:uri="012b183d-1ada-4ff6-b855-98c4d59bda2b"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -2164,20 +2175,9 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E55E6835-5439-4B85-9C34-8A416D678E4C}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C795275D-8D89-4504-820D-42600FA03DDE}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="c2ee6f6c-285d-4b95-ace0-9682ebe56039"/>
-    <ds:schemaRef ds:uri="012b183d-1ada-4ff6-b855-98c4d59bda2b"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
Erreur : site web inaccessible via HTTPS sur l'instance EC2
</commit_message>
<xml_diff>
--- a/Feuille de calcul de la base de connaissance-1.xlsx
+++ b/Feuille de calcul de la base de connaissance-1.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Anna\Documents\ODC\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E3742529-D561-49A7-8D9F-A635011B9630}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{18A21F2B-C531-4F79-8715-4EE8CA2F5E73}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="69" uniqueCount="65">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="78" uniqueCount="74">
   <si>
     <t>Commentaires</t>
   </si>
@@ -337,6 +337,37 @@
   </si>
   <si>
     <t>PB. 2</t>
+  </si>
+  <si>
+    <t>Instances Amazon EC2 (defi)</t>
+  </si>
+  <si>
+    <t>PB.3</t>
+  </si>
+  <si>
+    <t>Impossible d’accéder au site web de l’instance EC2 en utilisant HTTPS.</t>
+  </si>
+  <si>
+    <t>Le navigateur affiche "Ce site est inaccessible" lors de l’accès via https://IP-publique.
+Cependant, le site fonctionne avec http://IP-publique.</t>
+  </si>
+  <si>
+    <t>Le serveur web (httpd) est configuré uniquement pour HTTP (port 80) et non pour HTTPS (port 443).
+Aucun certificat SSL n’est configuré sur l’instance.</t>
+  </si>
+  <si>
+    <t>1. Vérifier que l’accès HTTP fonctionne.
+2. Utiliser HTTP au lieu de HTTPS si aucun certificat SSL n’est installé.</t>
+  </si>
+  <si>
+    <t>https://docs.aws.amazon.com/AWSEC2/latest/UserGuide/ec2-security-groups.html
+https://httpd.apache.org/docs/</t>
+  </si>
+  <si>
+    <t>HTTPS nécessite une configuration supplémentaire (certificat SSL). Par défaut, une instance EC2 avec httpd ne supporte que HTTP.</t>
+  </si>
+  <si>
+    <t>Prbleme 3</t>
   </si>
 </sst>
 </file>
@@ -600,7 +631,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="35">
+  <cellXfs count="36">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -671,13 +702,16 @@
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="6" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1034,13 +1068,13 @@
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.453125" defaultRowHeight="20"/>
   <cols>
     <col min="1" max="1" width="28.6328125" style="2" customWidth="1"/>
-    <col min="2" max="2" width="32.453125" style="3" customWidth="1"/>
+    <col min="2" max="2" width="34.54296875" style="3" customWidth="1"/>
     <col min="3" max="3" width="41.08984375" style="3" customWidth="1"/>
     <col min="4" max="4" width="130.1796875" style="2" customWidth="1"/>
-    <col min="5" max="5" width="118.08984375" style="2" customWidth="1"/>
+    <col min="5" max="5" width="148.54296875" style="2" customWidth="1"/>
     <col min="6" max="6" width="126.6328125" style="2" customWidth="1"/>
-    <col min="7" max="7" width="48" style="2" customWidth="1"/>
-    <col min="8" max="8" width="109" style="2" customWidth="1"/>
+    <col min="7" max="7" width="114.6328125" style="2" customWidth="1"/>
+    <col min="8" max="8" width="186.81640625" style="2" customWidth="1"/>
     <col min="9" max="9" width="61.6328125" style="2" customWidth="1"/>
     <col min="10" max="16384" width="11.453125" style="2"/>
   </cols>
@@ -1189,109 +1223,135 @@
       </c>
     </row>
     <row r="6" spans="1:9" ht="40.5" customHeight="1">
-      <c r="A6" s="29" t="s">
+      <c r="A6" s="30" t="s">
         <v>48</v>
       </c>
-      <c r="B6" s="32" t="s">
+      <c r="B6" s="33" t="s">
         <v>47</v>
       </c>
-      <c r="C6" s="34" t="s">
+      <c r="C6" s="35" t="s">
         <v>50</v>
       </c>
-      <c r="D6" s="26" t="s">
+      <c r="D6" s="25" t="s">
         <v>51</v>
       </c>
-      <c r="E6" s="26" t="s">
+      <c r="E6" s="25" t="s">
         <v>52</v>
       </c>
-      <c r="F6" s="26" t="s">
+      <c r="F6" s="25" t="s">
         <v>53</v>
       </c>
-      <c r="G6" s="26" t="s">
+      <c r="G6" s="25" t="s">
         <v>54</v>
       </c>
-      <c r="H6" s="26" t="s">
+      <c r="H6" s="25" t="s">
         <v>55</v>
       </c>
-      <c r="I6" s="27" t="s">
+      <c r="I6" s="28" t="s">
         <v>49</v>
       </c>
     </row>
     <row r="7" spans="1:9" ht="40" customHeight="1">
-      <c r="A7" s="30"/>
-      <c r="B7" s="33"/>
-      <c r="C7" s="31"/>
-      <c r="D7" s="24"/>
-      <c r="E7" s="24"/>
-      <c r="F7" s="24"/>
-      <c r="G7" s="24"/>
-      <c r="H7" s="24"/>
-      <c r="I7" s="28"/>
+      <c r="A7" s="31"/>
+      <c r="B7" s="34"/>
+      <c r="C7" s="32"/>
+      <c r="D7" s="26"/>
+      <c r="E7" s="26"/>
+      <c r="F7" s="26"/>
+      <c r="G7" s="26"/>
+      <c r="H7" s="26"/>
+      <c r="I7" s="29"/>
     </row>
     <row r="8" spans="1:9" ht="40" customHeight="1">
-      <c r="A8" s="30"/>
-      <c r="B8" s="33"/>
-      <c r="C8" s="31"/>
-      <c r="D8" s="24"/>
-      <c r="E8" s="24"/>
-      <c r="F8" s="24"/>
-      <c r="G8" s="24"/>
-      <c r="H8" s="24"/>
-      <c r="I8" s="28"/>
+      <c r="A8" s="31"/>
+      <c r="B8" s="34"/>
+      <c r="C8" s="32"/>
+      <c r="D8" s="26"/>
+      <c r="E8" s="26"/>
+      <c r="F8" s="26"/>
+      <c r="G8" s="26"/>
+      <c r="H8" s="26"/>
+      <c r="I8" s="29"/>
     </row>
     <row r="9" spans="1:9" ht="40" customHeight="1">
-      <c r="A9" s="25" t="s">
+      <c r="A9" s="27" t="s">
         <v>64</v>
       </c>
-      <c r="B9" s="31" t="s">
+      <c r="B9" s="32" t="s">
         <v>57</v>
       </c>
-      <c r="C9" s="31" t="s">
+      <c r="C9" s="32" t="s">
         <v>56</v>
       </c>
-      <c r="D9" s="24" t="s">
+      <c r="D9" s="26" t="s">
         <v>59</v>
       </c>
-      <c r="E9" s="24" t="s">
+      <c r="E9" s="26" t="s">
         <v>60</v>
       </c>
-      <c r="F9" s="24" t="s">
+      <c r="F9" s="26" t="s">
         <v>58</v>
       </c>
-      <c r="G9" s="24" t="s">
+      <c r="G9" s="26" t="s">
         <v>61</v>
       </c>
-      <c r="H9" s="24" t="s">
+      <c r="H9" s="26" t="s">
         <v>62</v>
       </c>
-      <c r="I9" s="24" t="s">
+      <c r="I9" s="29" t="s">
         <v>63</v>
       </c>
     </row>
     <row r="10" spans="1:9" ht="22.5" customHeight="1">
-      <c r="A10" s="25"/>
-      <c r="B10" s="31"/>
-      <c r="C10" s="31"/>
-      <c r="D10" s="24"/>
-      <c r="E10" s="24"/>
-      <c r="F10" s="24"/>
-      <c r="G10" s="24"/>
-      <c r="H10" s="24"/>
-      <c r="I10" s="24"/>
+      <c r="A10" s="27"/>
+      <c r="B10" s="32"/>
+      <c r="C10" s="32"/>
+      <c r="D10" s="26"/>
+      <c r="E10" s="26"/>
+      <c r="F10" s="26"/>
+      <c r="G10" s="26"/>
+      <c r="H10" s="26"/>
+      <c r="I10" s="29"/>
     </row>
     <row r="11" spans="1:9" ht="22.5" customHeight="1">
-      <c r="A11" s="25"/>
-      <c r="B11" s="31"/>
-      <c r="C11" s="31"/>
-      <c r="D11" s="24"/>
-      <c r="E11" s="24"/>
-      <c r="F11" s="24"/>
-      <c r="G11" s="24"/>
-      <c r="H11" s="24"/>
-      <c r="I11" s="24"/>
-    </row>
-    <row r="12" spans="1:9" ht="22.5">
-      <c r="A12" s="4"/>
+      <c r="A11" s="27"/>
+      <c r="B11" s="32"/>
+      <c r="C11" s="32"/>
+      <c r="D11" s="26"/>
+      <c r="E11" s="26"/>
+      <c r="F11" s="26"/>
+      <c r="G11" s="26"/>
+      <c r="H11" s="26"/>
+      <c r="I11" s="29"/>
+    </row>
+    <row r="12" spans="1:9" ht="60">
+      <c r="A12" s="4" t="s">
+        <v>66</v>
+      </c>
+      <c r="B12" s="3" t="s">
+        <v>65</v>
+      </c>
+      <c r="C12" s="3" t="s">
+        <v>67</v>
+      </c>
+      <c r="D12" s="3" t="s">
+        <v>68</v>
+      </c>
+      <c r="E12" s="3" t="s">
+        <v>69</v>
+      </c>
+      <c r="F12" s="3" t="s">
+        <v>70</v>
+      </c>
+      <c r="G12" s="3" t="s">
+        <v>71</v>
+      </c>
+      <c r="H12" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="I12" s="24" t="s">
+        <v>73</v>
+      </c>
     </row>
     <row r="13" spans="1:9" ht="22.5">
       <c r="A13" s="4"/>
@@ -1817,6 +1877,8 @@
     </row>
   </sheetData>
   <mergeCells count="18">
+    <mergeCell ref="D6:D8"/>
+    <mergeCell ref="E6:E8"/>
     <mergeCell ref="F6:F8"/>
     <mergeCell ref="G6:G8"/>
     <mergeCell ref="H9:H11"/>
@@ -1833,8 +1895,6 @@
     <mergeCell ref="G9:G11"/>
     <mergeCell ref="B6:B8"/>
     <mergeCell ref="C6:C8"/>
-    <mergeCell ref="D6:D8"/>
-    <mergeCell ref="E6:E8"/>
   </mergeCells>
   <phoneticPr fontId="13" type="noConversion"/>
   <dataValidations count="1">
@@ -1901,6 +1961,21 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Dokument" ma:contentTypeID="0x01010006807B066C556C4DA1F97EE96CC1104B" ma:contentTypeVersion="13" ma:contentTypeDescription="Utwórz nowy dokument." ma:contentTypeScope="" ma:versionID="cfb987611df5cdae7f7a5067c3395bc7">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="c2ee6f6c-285d-4b95-ace0-9682ebe56039" xmlns:ns3="012b183d-1ada-4ff6-b855-98c4d59bda2b" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="08f2586826dc5d0b05e832f2b79fc23a" ns2:_="" ns3:_="">
     <xsd:import namespace="c2ee6f6c-285d-4b95-ace0-9682ebe56039"/>
@@ -2123,36 +2198,10 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E55E6835-5439-4B85-9C34-8A416D678E4C}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C795275D-8D89-4504-820D-42600FA03DDE}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="c2ee6f6c-285d-4b95-ace0-9682ebe56039"/>
-    <ds:schemaRef ds:uri="012b183d-1ada-4ff6-b855-98c4d59bda2b"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -2175,9 +2224,20 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C795275D-8D89-4504-820D-42600FA03DDE}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E55E6835-5439-4B85-9C34-8A416D678E4C}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="c2ee6f6c-285d-4b95-ace0-9682ebe56039"/>
+    <ds:schemaRef ds:uri="012b183d-1ada-4ff6-b855-98c4d59bda2b"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
Amélioration possible : prévoir configuration HTTPS avec certificat SSL pour sécuriser l'accès
</commit_message>
<xml_diff>
--- a/Feuille de calcul de la base de connaissance-1.xlsx
+++ b/Feuille de calcul de la base de connaissance-1.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Anna\Documents\ODC\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9B3AA6BE-19D5-4489-BA34-CB700FB89955}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{43EC7823-6FB4-41EC-8BD5-D48A08D140E5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="8990" yWindow="100" windowWidth="10210" windowHeight="9980" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Entrées base de connaissances" sheetId="3" r:id="rId1"/>
@@ -711,13 +711,13 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="6" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1247,7 +1247,7 @@
       <c r="H6" s="25" t="s">
         <v>55</v>
       </c>
-      <c r="I6" s="28" t="s">
+      <c r="I6" s="29" t="s">
         <v>49</v>
       </c>
     </row>
@@ -1260,7 +1260,7 @@
       <c r="F7" s="26"/>
       <c r="G7" s="26"/>
       <c r="H7" s="26"/>
-      <c r="I7" s="29"/>
+      <c r="I7" s="27"/>
     </row>
     <row r="8" spans="1:9" ht="40" customHeight="1">
       <c r="A8" s="31"/>
@@ -1271,10 +1271,10 @@
       <c r="F8" s="26"/>
       <c r="G8" s="26"/>
       <c r="H8" s="26"/>
-      <c r="I8" s="29"/>
+      <c r="I8" s="27"/>
     </row>
     <row r="9" spans="1:9" ht="40" customHeight="1">
-      <c r="A9" s="27" t="s">
+      <c r="A9" s="28" t="s">
         <v>64</v>
       </c>
       <c r="B9" s="32" t="s">
@@ -1298,12 +1298,12 @@
       <c r="H9" s="26" t="s">
         <v>62</v>
       </c>
-      <c r="I9" s="29" t="s">
+      <c r="I9" s="27" t="s">
         <v>63</v>
       </c>
     </row>
     <row r="10" spans="1:9" ht="22.5" customHeight="1">
-      <c r="A10" s="27"/>
+      <c r="A10" s="28"/>
       <c r="B10" s="32"/>
       <c r="C10" s="32"/>
       <c r="D10" s="26"/>
@@ -1311,10 +1311,10 @@
       <c r="F10" s="26"/>
       <c r="G10" s="26"/>
       <c r="H10" s="26"/>
-      <c r="I10" s="29"/>
+      <c r="I10" s="27"/>
     </row>
     <row r="11" spans="1:9" ht="22.5" customHeight="1">
-      <c r="A11" s="27"/>
+      <c r="A11" s="28"/>
       <c r="B11" s="32"/>
       <c r="C11" s="32"/>
       <c r="D11" s="26"/>
@@ -1322,7 +1322,7 @@
       <c r="F11" s="26"/>
       <c r="G11" s="26"/>
       <c r="H11" s="26"/>
-      <c r="I11" s="29"/>
+      <c r="I11" s="27"/>
     </row>
     <row r="12" spans="1:9" ht="60">
       <c r="A12" s="4" t="s">
@@ -1877,11 +1877,6 @@
     </row>
   </sheetData>
   <mergeCells count="18">
-    <mergeCell ref="D6:D8"/>
-    <mergeCell ref="E6:E8"/>
-    <mergeCell ref="F6:F8"/>
-    <mergeCell ref="G6:G8"/>
-    <mergeCell ref="H9:H11"/>
     <mergeCell ref="I9:I11"/>
     <mergeCell ref="A9:A11"/>
     <mergeCell ref="H6:H8"/>
@@ -1895,6 +1890,11 @@
     <mergeCell ref="G9:G11"/>
     <mergeCell ref="B6:B8"/>
     <mergeCell ref="C6:C8"/>
+    <mergeCell ref="D6:D8"/>
+    <mergeCell ref="E6:E8"/>
+    <mergeCell ref="F6:F8"/>
+    <mergeCell ref="G6:G8"/>
+    <mergeCell ref="H9:H11"/>
   </mergeCells>
   <phoneticPr fontId="13" type="noConversion"/>
   <dataValidations count="1">
@@ -1961,21 +1961,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Dokument" ma:contentTypeID="0x01010006807B066C556C4DA1F97EE96CC1104B" ma:contentTypeVersion="13" ma:contentTypeDescription="Utwórz nowy dokument." ma:contentTypeScope="" ma:versionID="cfb987611df5cdae7f7a5067c3395bc7">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="c2ee6f6c-285d-4b95-ace0-9682ebe56039" xmlns:ns3="012b183d-1ada-4ff6-b855-98c4d59bda2b" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="08f2586826dc5d0b05e832f2b79fc23a" ns2:_="" ns3:_="">
     <xsd:import namespace="c2ee6f6c-285d-4b95-ace0-9682ebe56039"/>
@@ -2198,10 +2183,36 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C795275D-8D89-4504-820D-42600FA03DDE}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E55E6835-5439-4B85-9C34-8A416D678E4C}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="c2ee6f6c-285d-4b95-ace0-9682ebe56039"/>
+    <ds:schemaRef ds:uri="012b183d-1ada-4ff6-b855-98c4d59bda2b"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -2224,20 +2235,9 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E55E6835-5439-4B85-9C34-8A416D678E4C}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C795275D-8D89-4504-820D-42600FA03DDE}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="c2ee6f6c-285d-4b95-ace0-9682ebe56039"/>
-    <ds:schemaRef ds:uri="012b183d-1ada-4ff6-b855-98c4d59bda2b"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>